<commit_message>
Modification sur le narratif 5e3109504b71c77dd1766e21e0e291512f99e9a7
</commit_message>
<xml_diff>
--- a/nmoreau/ig/CodeSystem-document-type-code-system.xlsx
+++ b/nmoreau/ig/CodeSystem-document-type-code-system.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="59">
   <si>
     <t>Property</t>
   </si>
@@ -36,7 +36,7 @@
     <t>Name</t>
   </si>
   <si>
-    <t>PreadmissionCodeSystemDocumentTypeFr</t>
+    <t>PreadmissionDocumentTypeCodeSystem</t>
   </si>
   <si>
     <t>Title</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>active</t>
+    <t>draft</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-24T12:53:37+00:00</t>
+    <t>2025-04-25T09:56:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -120,7 +120,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>13</t>
+    <t>9</t>
   </si>
   <si>
     <t>Level</t>
@@ -138,19 +138,13 @@
     <t>1</t>
   </si>
   <si>
-    <t>CNI</t>
-  </si>
-  <si>
-    <t>Carte d’identité</t>
-  </si>
-  <si>
-    <t>CNI_RECTO</t>
+    <t>CN_RECTO</t>
   </si>
   <si>
     <t>Recto Carte d’identité</t>
   </si>
   <si>
-    <t>CNI_VERSO</t>
+    <t>CN_VERSO</t>
   </si>
   <si>
     <t>Verso Carte d’identité</t>
@@ -162,12 +156,6 @@
     <t>Carte Vitale</t>
   </si>
   <si>
-    <t>PASSPORT</t>
-  </si>
-  <si>
-    <t>Passeport</t>
-  </si>
-  <si>
     <t>JUSTIFICATIF_ID</t>
   </si>
   <si>
@@ -192,22 +180,10 @@
     <t>Verso Carte mutuelle</t>
   </si>
   <si>
-    <t>LIVRET</t>
-  </si>
-  <si>
-    <t>Livret de famille</t>
-  </si>
-  <si>
     <t>JUSTIFICATIF_DOM</t>
   </si>
   <si>
     <t>Justificatif de domicile</t>
-  </si>
-  <si>
-    <t>CARTE_SEJOUR</t>
-  </si>
-  <si>
-    <t>Carte de séjour</t>
   </si>
   <si>
     <t>ARRET_TRAVAIL</t>
@@ -527,7 +503,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -652,54 +628,6 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11">
-      <c r="A11" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B11" t="s" s="2">
-        <v>59</v>
-      </c>
-      <c r="C11" t="s" s="2">
-        <v>60</v>
-      </c>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B12" t="s" s="2">
-        <v>61</v>
-      </c>
-      <c r="C12" t="s" s="2">
-        <v>62</v>
-      </c>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B13" t="s" s="2">
-        <v>63</v>
-      </c>
-      <c r="C13" t="s" s="2">
-        <v>64</v>
-      </c>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B14" t="s" s="2">
-        <v>65</v>
-      </c>
-      <c r="C14" t="s" s="2">
-        <v>66</v>
-      </c>
-      <c r="D14" s="2"/>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Corrections demandées en PR + travail sur les consentements 73ecd155f37082c1022e70700cc5d08ed369625d
</commit_message>
<xml_diff>
--- a/nmoreau/ig/CodeSystem-document-type-code-system.xlsx
+++ b/nmoreau/ig/CodeSystem-document-type-code-system.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="60">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-28T10:41:02+00:00</t>
+    <t>2025-05-05T08:51:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -453,7 +453,9 @@
       <c r="A16" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="B16" s="2"/>
+      <c r="B16" t="s" s="2">
+        <v>13</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">

</xml_diff>

<commit_message>
Déplacement du narratif sur les ressources dans les pages de conformité en tant qu'introduction 00c8e39ccc487ca393c42ed1e9b2cde74c8c52b8
</commit_message>
<xml_diff>
--- a/nmoreau/ig/CodeSystem-document-type-code-system.xlsx
+++ b/nmoreau/ig/CodeSystem-document-type-code-system.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-06T13:54:59+00:00</t>
+    <t>2025-05-14T09:00:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Interop'Santé (http://interopsante.org/)</t>
   </si>
   <si>
-    <t>InteropSanté (fhir@interopsante.org(work))</t>
+    <t>InteropSanté (fhir@interopsante.org(Work))</t>
   </si>
   <si>
     <t>Jurisdiction</t>

</xml_diff>